<commit_message>
Refresh Rick Tesla V1 live listings
</commit_message>
<xml_diff>
--- a/publish/tesla-parts-sniper-v1-workbench/downloads/tesla-parts-sniper-v1-google-sheet.xlsx
+++ b/publish/tesla-parts-sniper-v1-workbench/downloads/tesla-parts-sniper-v1-google-sheet.xlsx
@@ -183,7 +183,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:55+00:00</t>
+          <t>2026-05-01T11:31:20+00:00</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -260,7 +260,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:18+00:00</t>
+          <t>2026-05-01T11:31:41+00:00</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -337,7 +337,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:53+00:00</t>
+          <t>2026-05-01T11:32:04+00:00</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -414,7 +414,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:19+00:00</t>
+          <t>2026-05-01T11:32:31+00:00</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -491,7 +491,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:44+00:00</t>
+          <t>2026-05-01T11:32:51+00:00</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:29+00:00</t>
+          <t>2026-05-01T11:33:30+00:00</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:59+00:00</t>
+          <t>2026-05-01T11:31:24+00:00</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:02+00:00</t>
+          <t>2026-05-01T11:31:27+00:00</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:07+00:00</t>
+          <t>2026-05-01T11:31:31+00:00</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:11+00:00</t>
+          <t>2026-05-01T11:31:34+00:00</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:14+00:00</t>
+          <t>2026-05-01T11:31:37+00:00</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:18+00:00</t>
+          <t>2026-05-01T11:31:40+00:00</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:22+00:00</t>
+          <t>2026-05-01T11:31:44+00:00</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:25+00:00</t>
+          <t>2026-05-01T11:31:47+00:00</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:30+00:00</t>
+          <t>2026-05-01T11:31:53+00:00</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:33+00:00</t>
+          <t>2026-05-01T11:31:56+00:00</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:48+00:00</t>
+          <t>2026-05-01T11:32:00+00:00</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:52+00:00</t>
+          <t>2026-05-01T11:32:03+00:00</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:56+00:00</t>
+          <t>2026-05-01T11:32:07+00:00</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:59+00:00</t>
+          <t>2026-05-01T11:32:10+00:00</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:03+00:00</t>
+          <t>2026-05-01T11:32:19+00:00</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:13+00:00</t>
+          <t>2026-05-01T11:32:23+00:00</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:16+00:00</t>
+          <t>2026-05-01T11:32:27+00:00</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:19+00:00</t>
+          <t>2026-05-01T11:32:31+00:00</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:25+00:00</t>
+          <t>2026-05-01T11:32:34+00:00</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:29+00:00</t>
+          <t>2026-05-01T11:32:38+00:00</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:32+00:00</t>
+          <t>2026-05-01T11:32:41+00:00</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:36+00:00</t>
+          <t>2026-05-01T11:32:44+00:00</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:39+00:00</t>
+          <t>2026-05-01T11:32:47+00:00</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:43+00:00</t>
+          <t>2026-05-01T11:32:50+00:00</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:46+00:00</t>
+          <t>2026-05-01T11:32:54+00:00</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:49+00:00</t>
+          <t>2026-05-01T11:32:57+00:00</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:54+00:00</t>
+          <t>2026-05-01T11:33:01+00:00</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:58+00:00</t>
+          <t>2026-05-01T11:33:04+00:00</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:01+00:00</t>
+          <t>2026-05-01T11:33:07+00:00</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:04+00:00</t>
+          <t>2026-05-01T11:33:10+00:00</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:32+00:00</t>
+          <t>2026-05-01T11:33:33+00:00</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:35+00:00</t>
+          <t>2026-05-01T11:33:36+00:00</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:40+00:00</t>
+          <t>2026-05-01T11:33:40+00:00</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:44+00:00</t>
+          <t>2026-05-01T11:33:44+00:00</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:52+00:00</t>
+          <t>2026-05-01T11:33:47+00:00</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:55+00:00</t>
+          <t>2026-05-01T11:33:50+00:00</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:18+00:00</t>
+          <t>2026-05-01T11:31:40+00:00</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:52+00:00</t>
+          <t>2026-05-01T11:32:03+00:00</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:19+00:00</t>
+          <t>2026-05-01T11:32:31+00:00</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3648,7 +3648,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:43+00:00</t>
+          <t>2026-05-01T11:32:50+00:00</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:04+00:00</t>
+          <t>2026-05-01T11:33:10+00:00</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:55+00:00</t>
+          <t>2026-05-01T11:33:50+00:00</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:18+00:00</t>
+          <t>2026-05-01T11:31:40+00:00</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:52+00:00</t>
+          <t>2026-05-01T11:32:03+00:00</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:19+00:00</t>
+          <t>2026-05-01T11:32:31+00:00</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:43+00:00</t>
+          <t>2026-05-01T11:32:50+00:00</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:04+00:00</t>
+          <t>2026-05-01T11:33:10+00:00</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:55+00:00</t>
+          <t>2026-05-01T11:33:50+00:00</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:18+00:00</t>
+          <t>2026-05-01T11:31:40+00:00</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4418,7 +4418,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:52+00:00</t>
+          <t>2026-05-01T11:32:03+00:00</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:19+00:00</t>
+          <t>2026-05-01T11:32:31+00:00</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:43+00:00</t>
+          <t>2026-05-01T11:32:50+00:00</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -4649,7 +4649,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:04+00:00</t>
+          <t>2026-05-01T11:33:10+00:00</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:55+00:00</t>
+          <t>2026-05-01T11:33:50+00:00</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -4803,7 +4803,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:18+00:00</t>
+          <t>2026-05-01T11:31:40+00:00</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>2026-05-01T09:50:52+00:00</t>
+          <t>2026-05-01T11:32:03+00:00</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -4957,7 +4957,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:19+00:00</t>
+          <t>2026-05-01T11:32:31+00:00</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>2026-05-01T09:51:43+00:00</t>
+          <t>2026-05-01T11:32:50+00:00</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:04+00:00</t>
+          <t>2026-05-01T11:33:10+00:00</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -5188,7 +5188,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:55+00:00</t>
+          <t>2026-05-01T11:33:50+00:00</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:10+00:00</t>
+          <t>2026-05-01T11:35:14+00:00</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:33+00:00</t>
+          <t>2026-05-01T11:35:37+00:00</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -5384,7 +5384,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>seattle / 7h ago NE Portland</t>
+          <t>seattle / 8h ago NE Portland</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:33+00:00</t>
+          <t>2026-05-01T11:35:37+00:00</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -5496,7 +5496,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:55+00:00</t>
+          <t>2026-05-01T11:35:59+00:00</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -5573,7 +5573,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:03+00:00</t>
+          <t>2026-05-01T11:36:08+00:00</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:18+00:00</t>
+          <t>2026-05-01T11:36:22+00:00</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:18+00:00</t>
+          <t>2026-05-01T11:36:22+00:00</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:30+00:00</t>
+          <t>2026-05-01T11:30:56+00:00</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -5881,7 +5881,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:04+00:00</t>
+          <t>2026-05-01T11:33:10+00:00</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:55+00:00</t>
+          <t>2026-05-01T11:33:50+00:00</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -6035,7 +6035,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:23+00:00</t>
+          <t>2026-05-01T11:34:13+00:00</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -6112,7 +6112,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:45+00:00</t>
+          <t>2026-05-01T11:34:48+00:00</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -6189,7 +6189,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:05+00:00</t>
+          <t>2026-05-01T11:35:11+00:00</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -6266,7 +6266,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:30+00:00</t>
+          <t>2026-05-01T11:35:32+00:00</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:52+00:00</t>
+          <t>2026-05-01T11:35:55+00:00</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:14+00:00</t>
+          <t>2026-05-01T11:36:18+00:00</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:39+00:00</t>
+          <t>2026-05-01T11:36:38+00:00</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -6574,7 +6574,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:35+00:00</t>
+          <t>2026-05-01T11:31:00+00:00</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -6651,7 +6651,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:38+00:00</t>
+          <t>2026-05-01T11:31:04+00:00</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:42+00:00</t>
+          <t>2026-05-01T11:31:08+00:00</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:47+00:00</t>
+          <t>2026-05-01T11:31:12+00:00</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -6882,7 +6882,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:50+00:00</t>
+          <t>2026-05-01T11:31:16+00:00</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:54+00:00</t>
+          <t>2026-05-01T11:31:20+00:00</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:10+00:00</t>
+          <t>2026-05-01T11:33:13+00:00</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -7113,7 +7113,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:13+00:00</t>
+          <t>2026-05-01T11:33:17+00:00</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -7190,7 +7190,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:18+00:00</t>
+          <t>2026-05-01T11:33:20+00:00</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -7267,7 +7267,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:22+00:00</t>
+          <t>2026-05-01T11:33:23+00:00</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -7344,7 +7344,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:25+00:00</t>
+          <t>2026-05-01T11:33:26+00:00</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -7421,7 +7421,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:28+00:00</t>
+          <t>2026-05-01T11:33:29+00:00</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -7498,7 +7498,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:58+00:00</t>
+          <t>2026-05-01T11:33:54+00:00</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -7575,7 +7575,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:02+00:00</t>
+          <t>2026-05-01T11:33:57+00:00</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:06+00:00</t>
+          <t>2026-05-01T11:33:59+00:00</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -7729,7 +7729,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:15+00:00</t>
+          <t>2026-05-01T11:34:06+00:00</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:19+00:00</t>
+          <t>2026-05-01T11:34:09+00:00</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:23+00:00</t>
+          <t>2026-05-01T11:34:12+00:00</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -7915,7 +7915,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>No live Craigslist result found yet: Tesla Model Y front bumper in spokane</t>
+          <t>No live Craigslist result found yet: Tesla Model Y front bumper in eugene</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -7925,7 +7925,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>spokane</t>
+          <t>eugene</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -7955,12 +7955,12 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://spokane.craigslist.org/search/pta?query=Tesla+Model+Y+front+bumper</t>
+          <t>https://eugene.craigslist.org/search/pta?query=Tesla+Model+Y+front+bumper</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:31+00:00</t>
+          <t>2026-05-01T11:34:42+00:00</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>No live Craigslist result found yet: Tesla Model Y front bumper in eugene</t>
+          <t>No live Craigslist result found yet: Tesla Model Y front bumper in bend</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -8002,7 +8002,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>eugene</t>
+          <t>bend</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -8032,12 +8032,12 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>https://eugene.craigslist.org/search/pta?query=Tesla+Model+Y+front+bumper</t>
+          <t>https://bend.craigslist.org/search/pta?query=Tesla+Model+Y+front+bumper</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:41+00:00</t>
+          <t>2026-05-01T11:34:47+00:00</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -8069,7 +8069,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>No live Craigslist result found yet: Tesla Model Y front bumper in bend</t>
+          <t>No live Craigslist result found yet: Tesla Model Y rear bumper in eugene</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>bend</t>
+          <t>eugene</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -8089,7 +8089,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>front bumper</t>
+          <t>rear bumper</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -8109,12 +8109,12 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>https://bend.craigslist.org/search/pta?query=Tesla+Model+Y+front+bumper</t>
+          <t>https://eugene.craigslist.org/search/pta?query=Tesla+Model+Y+rear+bumper</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:45+00:00</t>
+          <t>2026-05-01T11:35:07+00:00</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -8146,7 +8146,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>No live Craigslist result found yet: Tesla Model Y rear bumper in spokane</t>
+          <t>No live Craigslist result found yet: Tesla Model Y rear bumper in bend</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -8156,7 +8156,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>spokane</t>
+          <t>bend</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -8186,12 +8186,12 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>https://spokane.craigslist.org/search/pta?query=Tesla+Model+Y+rear+bumper</t>
+          <t>https://bend.craigslist.org/search/pta?query=Tesla+Model+Y+rear+bumper</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:51+00:00</t>
+          <t>2026-05-01T11:35:10+00:00</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>No live Craigslist result found yet: Tesla Model Y rear bumper in eugene</t>
+          <t>No live Craigslist result found yet: Tesla Model Y headlight in spokane</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>eugene</t>
+          <t>spokane</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -8243,7 +8243,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>rear bumper</t>
+          <t>headlight</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -8263,12 +8263,12 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>https://eugene.craigslist.org/search/pta?query=Tesla+Model+Y+rear+bumper</t>
+          <t>https://spokane.craigslist.org/search/pta?query=Tesla+Model+Y+headlight</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:01+00:00</t>
+          <t>2026-05-01T11:35:17+00:00</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -8300,7 +8300,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>No live Craigslist result found yet: Tesla Model Y rear bumper in bend</t>
+          <t>No live Craigslist result found yet: Tesla Model Y door in spokane</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -8310,7 +8310,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>bend</t>
+          <t>spokane</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -8320,7 +8320,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>rear bumper</t>
+          <t>door</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -8340,12 +8340,12 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>https://bend.craigslist.org/search/pta?query=Tesla+Model+Y+rear+bumper</t>
+          <t>https://spokane.craigslist.org/search/pta?query=Tesla+Model+Y+door</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:04+00:00</t>
+          <t>2026-05-01T11:35:40+00:00</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -8377,7 +8377,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>No live Craigslist result found yet: Tesla Model Y headlight in spokane</t>
+          <t>No live Craigslist result found yet: Tesla Model Y wheel in bend</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>spokane</t>
+          <t>bend</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -8397,7 +8397,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>headlight</t>
+          <t>wheel</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -8417,12 +8417,12 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>https://spokane.craigslist.org/search/pta?query=Tesla+Model+Y+headlight</t>
+          <t>https://bend.craigslist.org/search/pta?query=Tesla+Model+Y+wheel</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:13+00:00</t>
+          <t>2026-05-01T11:36:18+00:00</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>No live Craigslist result found yet: Tesla Model 3 front bumper in seattle</t>
+          <t>No live Craigslist result found yet: Tesla Model 3 hood in bellingham</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>seattle</t>
+          <t>bellingham</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -8474,7 +8474,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>front bumper</t>
+          <t>hood</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -8494,12 +8494,12 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/search/pta?query=Tesla+Model+3+front+bumper</t>
+          <t>https://bellingham.craigslist.org/search/pta?query=Tesla+Model+3+hood</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:45+00:00</t>
+          <t>2026-05-01T11:36:26+00:00</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -8531,7 +8531,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>No live Craigslist result found yet: Tesla Model 3 front bumper in eugene</t>
+          <t>No live Craigslist result found yet: Tesla Model 3 hood in bend</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -8541,7 +8541,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>eugene</t>
+          <t>bend</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -8551,7 +8551,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>front bumper</t>
+          <t>hood</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -8571,12 +8571,12 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://eugene.craigslist.org/search/pta?query=Tesla+Model+3+front+bumper</t>
+          <t>https://bend.craigslist.org/search/pta?query=Tesla+Model+3+hood</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:58+00:00</t>
+          <t>2026-05-01T11:36:38+00:00</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -8608,7 +8608,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>No live Craigslist result found yet: Tesla Model 3 front bumper in bend</t>
+          <t>No live Craigslist result found yet: Tesla Model 3 front bumper in bellingham</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -8618,7 +8618,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>bend</t>
+          <t>bellingham</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -8648,12 +8648,12 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>https://bend.craigslist.org/search/pta?query=Tesla+Model+3+front+bumper</t>
+          <t>https://bellingham.craigslist.org/search/pta?query=Tesla+Model+3+front+bumper</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>2026-05-01T09:56:02+00:00</t>
+          <t>2026-05-01T11:36:51+00:00</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -8680,12 +8680,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Car-Part.com</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Car-Part usable result workflow: Tesla 2024 Model Y hood</t>
+          <t>No live Craigslist result found yet: Tesla Model 3 front bumper in eugene</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -8695,17 +8695,17 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Nationwide / Car-Part</t>
+          <t>eugene</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2024 Tesla Model Y</t>
+          <t> Tesla Model 3</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>hood</t>
+          <t>front bumper</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -8725,17 +8725,17 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://www.car-part.com/cgi-bin/search.cgi?userSearch=int&amp;userPart=Tesla+2024+Model+Y+hood</t>
+          <t>https://eugene.craigslist.org/search/pta?query=Tesla+Model+3+front+bumper</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:54+00:00</t>
+          <t>2026-05-01T11:36:59+00:00</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>68</t>
         </is>
       </c>
       <c r="M113" t="inlineStr">
@@ -8750,19 +8750,19 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>year match, model match, part match, direct link, manual review source; manual review/no automated outreach</t>
+          <t>year match, model match, part match, direct link, public source; manual review/no automated outreach</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Car-Part.com</t>
+          <t>Craigslist</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Car-Part usable result workflow: Tesla 2024 Model Y front bumper</t>
+          <t>No live Craigslist result found yet: Tesla Model 3 front bumper in bend</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -8772,12 +8772,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Nationwide / Car-Part</t>
+          <t>bend</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2024 Tesla Model Y</t>
+          <t> Tesla Model 3</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -8802,17 +8802,17 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>https://www.car-part.com/cgi-bin/search.cgi?userSearch=int&amp;userPart=Tesla+2024+Model+Y+front+bumper</t>
+          <t>https://bend.craigslist.org/search/pta?query=Tesla+Model+3+front+bumper</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:28+00:00</t>
+          <t>2026-05-01T11:37:02+00:00</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>68</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
@@ -8827,19 +8827,19 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>year match, model match, part match, direct link, manual review source; manual review/no automated outreach</t>
+          <t>year match, model match, part match, direct link, public source; manual review/no automated outreach</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Car-Part.com</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Manual review search: Tesla 2024 Model Y hood</t>
+          <t>Car-Part usable result workflow: Tesla 2024 Model Y hood</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -8849,7 +8849,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>West Coast</t>
+          <t>Nationwide / Car-Part</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -8879,12 +8879,12 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://www.copart.com/lotSearchResults?free=true&amp;query=Tesla+2024+Model+Y+hood</t>
+          <t>https://www.car-part.com/cgi-bin/search.cgi?userSearch=int&amp;userPart=Tesla+2024+Model+Y+hood</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:54+00:00</t>
+          <t>2026-05-01T11:31:20+00:00</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -8911,12 +8911,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Car-Part.com</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Manual review search: Tesla 2024 Model Y front bumper</t>
+          <t>Car-Part usable result workflow: Tesla 2024 Model Y front bumper</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -8926,7 +8926,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>West Coast</t>
+          <t>Nationwide / Car-Part</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -8956,12 +8956,12 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>https://www.copart.com/lotSearchResults?free=true&amp;query=Tesla+2024+Model+Y+front+bumper</t>
+          <t>https://www.car-part.com/cgi-bin/search.cgi?userSearch=int&amp;userPart=Tesla+2024+Model+Y+front+bumper</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:28+00:00</t>
+          <t>2026-05-01T11:33:29+00:00</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -8988,7 +8988,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Facebook Marketplace</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -9033,12 +9033,12 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/search/?query=Tesla%25202024%2520Model%2520Y%2520hood</t>
+          <t>https://www.copart.com/lotSearchResults?free=true&amp;query=Tesla+2024+Model+Y+hood</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:54+00:00</t>
+          <t>2026-05-01T11:31:20+00:00</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -9065,7 +9065,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Facebook Marketplace</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -9110,12 +9110,12 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/search/?query=Tesla%25202024%2520Model%2520Y%2520front%2520bumper</t>
+          <t>https://www.copart.com/lotSearchResults?free=true&amp;query=Tesla+2024+Model+Y+front+bumper</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:28+00:00</t>
+          <t>2026-05-01T11:33:29+00:00</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -9142,7 +9142,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>IAAI</t>
+          <t>Facebook Marketplace</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -9187,12 +9187,12 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://www.iaai.com/Search?Keyword=Tesla+2024+Model+Y+hood</t>
+          <t>https://www.facebook.com/marketplace/search/?query=Tesla%25202024%2520Model%2520Y%2520hood</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>2026-05-01T09:49:54+00:00</t>
+          <t>2026-05-01T11:31:20+00:00</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -9219,7 +9219,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>IAAI</t>
+          <t>Facebook Marketplace</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -9264,12 +9264,12 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>https://www.iaai.com/Search?Keyword=Tesla+2024+Model+Y+front+bumper</t>
+          <t>https://www.facebook.com/marketplace/search/?query=Tesla%25202024%2520Model%2520Y%2520front%2520bumper</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>2026-05-01T09:52:28+00:00</t>
+          <t>2026-05-01T11:33:29+00:00</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -9296,32 +9296,32 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>IAAI</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Tesla model 3 or Y headlight Left side</t>
+          <t>Manual review search: Tesla 2024 Model Y hood</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>$350</t>
+          <t/>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>seattle / Milwaukie</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t> Tesla Model Y</t>
+          <t>2024 Tesla Model Y</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>headlight</t>
+          <t>hood</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -9341,17 +9341,17 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-or-headlight-left/7929779630.html</t>
+          <t>https://www.iaai.com/Search?Keyword=Tesla+2024+Model+Y+hood</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:10+00:00</t>
+          <t>2026-05-01T11:31:20+00:00</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>63</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
@@ -9361,44 +9361,44 @@
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>Watchlist</t>
+          <t>Manual Review</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>year match, part match, price visible, direct link, public source</t>
+          <t>year match, model match, part match, direct link, manual review source; manual review/no automated outreach</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Craigslist</t>
+          <t>IAAI</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Tesla half yolk steering wheel</t>
+          <t>Manual review search: Tesla 2024 Model Y front bumper</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>$200</t>
+          <t/>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>seattle / Seattle</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t> Tesla Model Y</t>
+          <t>2024 Tesla Model Y</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>wheel</t>
+          <t>front bumper</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -9418,17 +9418,17 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/see/pts/d/tesla-half-yolk-steering-wheel/7930743561.html</t>
+          <t>https://www.iaai.com/Search?Keyword=Tesla+2024+Model+Y+front+bumper</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:55+00:00</t>
+          <t>2026-05-01T11:33:29+00:00</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>63</t>
         </is>
       </c>
       <c r="M122" t="inlineStr">
@@ -9438,12 +9438,12 @@
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t>Watchlist</t>
+          <t>Manual Review</t>
         </is>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>year match, part match, price visible, direct link, public source</t>
+          <t>year match, model match, part match, direct link, manual review source; manual review/no automated outreach</t>
         </is>
       </c>
     </row>
@@ -9455,17 +9455,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Tesla Model Y 3 Parts</t>
+          <t>Tesla model 3 or Y headlight Left side</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t/>
+          <t>$350</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>seattle / Marysville</t>
+          <t>seattle / Milwaukie</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -9475,7 +9475,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>front bumper</t>
+          <t>headlight</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -9495,17 +9495,17 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-3-parts/7921311562.html</t>
+          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-or-headlight-left/7929779630.html</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:26+00:00</t>
+          <t>2026-05-01T11:35:14+00:00</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>53</t>
         </is>
       </c>
       <c r="M123" t="inlineStr">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>year match, model match, direct link, public source</t>
+          <t>year match, part match, price visible, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -9532,17 +9532,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Tesla Model Y Left Headlight (New)</t>
+          <t>Tesla half yolk steering wheel</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>$250</t>
+          <t>$200</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>bellingham / north vancouver</t>
+          <t>seattle / Seattle</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>headlight</t>
+          <t>wheel</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -9572,32 +9572,32 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>https://vancouver.craigslist.org/nvn/pts/d/north-vancouver-tesla-model-left/7896365226.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/tesla-half-yolk-steering-wheel/7930743561.html</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:19+00:00</t>
+          <t>2026-05-01T11:35:59+00:00</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>53</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>Duplicate</t>
+          <t>Watchlist</t>
         </is>
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>year match, model match, part match, price visible, direct link, public source</t>
+          <t>year match, part match, price visible, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -9609,17 +9609,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Tesla Model Y Door Wiring Rear Right 2020-2024 OEM 1489</t>
+          <t>Tesla Model Y 3 Parts</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>$135</t>
+          <t/>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>spokane / Marysville</t>
+          <t>seattle / Marysville</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -9629,7 +9629,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>door</t>
+          <t>front bumper</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -9649,32 +9649,32 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-door-wiring-rear/7922263989.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-3-parts/7921311562.html</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:36+00:00</t>
+          <t>2026-05-01T11:34:18+00:00</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>43</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>Duplicate</t>
+          <t>Watchlist</t>
         </is>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>year match, model match, part match, price visible, direct link, public source</t>
+          <t>year match, model match, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -9686,17 +9686,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Tesla Model Y Door Wiring Rear Right 2020-2024 OEM 1489</t>
+          <t>Tesla Model Y Left Headlight (New)</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>$135</t>
+          <t>$250</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>bellingham / Marysville</t>
+          <t>bellingham / north vancouver</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>door</t>
+          <t>headlight</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -9726,12 +9726,12 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-door-wiring-rear/7922263989.html</t>
+          <t>https://vancouver.craigslist.org/nvn/pts/d/north-vancouver-tesla-model-left/7896365226.html</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:40+00:00</t>
+          <t>2026-05-01T11:35:21+00:00</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -9763,17 +9763,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2021-2023 Tesla Model Y Front Drivers Left Door Panel Card</t>
+          <t>Tesla Model Y Door Wiring Rear Right 2020-2024 OEM 1489</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>$100</t>
+          <t>$135</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>bellingham / 7h ago NE Portland</t>
+          <t>bellingham / Marysville</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -9803,12 +9803,12 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-front-drivers-left/7917863484.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-door-wiring-rear/7922263989.html</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:40+00:00</t>
+          <t>2026-05-01T11:35:44+00:00</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -9850,7 +9850,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>portland / 7h ago NE Portland</t>
+          <t>bellingham / 8h ago NE Portland</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -9885,7 +9885,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:43+00:00</t>
+          <t>2026-05-01T11:35:44+00:00</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -9917,17 +9917,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Tesla Model Y Door Wiring Rear Right 2020-2024 OEM 1489</t>
+          <t>2021-2023 Tesla Model Y Front Drivers Left Door Panel Card</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>$135</t>
+          <t>$100</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>portland / Marysville</t>
+          <t>portland / 8h ago NE Portland</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -9957,12 +9957,12 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-door-wiring-rear/7922263989.html</t>
+          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-front-drivers-left/7917863484.html</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:43+00:00</t>
+          <t>2026-05-01T11:35:48+00:00</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -9994,17 +9994,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2021-2023 Tesla Model Y Front Drivers Left Door Panel Card</t>
+          <t>Tesla Model Y Door Wiring Rear Right 2020-2024 OEM 1489</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>$100</t>
+          <t>$135</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>eugene / 7h ago NE Portland</t>
+          <t>portland / Marysville</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -10034,12 +10034,12 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-front-drivers-left/7917863484.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-door-wiring-rear/7922263989.html</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:48+00:00</t>
+          <t>2026-05-01T11:35:48+00:00</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -10081,7 +10081,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>bend / 7h ago NE Portland</t>
+          <t>eugene / 8h ago NE Portland</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -10116,7 +10116,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:52+00:00</t>
+          <t>2026-05-01T11:35:51+00:00</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -10148,17 +10148,17 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Tesla Model Y performance 21” wheel rims covers curb protectors gunmetal grey</t>
+          <t>2021-2023 Tesla Model Y Front Drivers Left Door Panel Card</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>$79</t>
+          <t>$100</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>bellingham / Vancouver</t>
+          <t>bend / 8h ago NE Portland</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -10168,7 +10168,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>wheel</t>
+          <t>door</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -10188,12 +10188,12 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>https://vancouver.craigslist.org/van/pts/d/vancouver-tesla-model-performance-21/7901293693.html</t>
+          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-front-drivers-left/7917863484.html</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:03+00:00</t>
+          <t>2026-05-01T11:35:55+00:00</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -10225,27 +10225,27 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Tesla Model 3 Clear PPF Hood, fenders, headlights, mirrors fog lights</t>
+          <t>Tesla Model Y performance 21” wheel rims covers curb protectors gunmetal grey</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>$229</t>
+          <t>$79</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>spokane / Tukwila</t>
+          <t>bellingham / Vancouver</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t> Tesla Model 3</t>
+          <t> Tesla Model Y</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>hood</t>
+          <t>wheel</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -10265,12 +10265,12 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/skc/pts/d/seattle-tesla-model-clear-ppf-hood/7917727783.html</t>
+          <t>https://vancouver.craigslist.org/van/pts/d/vancouver-tesla-model-performance-21/7901293693.html</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:22+00:00</t>
+          <t>2026-05-01T11:36:08+00:00</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
@@ -10312,7 +10312,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>bellingham / Tukwila</t>
+          <t>spokane / Tukwila</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -10347,7 +10347,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:26+00:00</t>
+          <t>2026-05-01T11:36:25+00:00</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -10389,7 +10389,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>bellingham / clark/cowlitz WA</t>
+          <t>portland / clark/cowlitz WA</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -10424,7 +10424,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:26+00:00</t>
+          <t>2026-05-01T11:36:30+00:00</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -10456,17 +10456,17 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>NEW 2017 2022 2023 Pair TESLA MODEL 3 FRONT LEFT RIGHT Side HOOD HINGE</t>
+          <t>Tesla Model 3 Clear PPF Hood, fenders, headlights, mirrors fog lights</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>$80</t>
+          <t>$229</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>portland / clark/cowlitz WA</t>
+          <t>portland / Tukwila</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -10496,12 +10496,12 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>https://portland.craigslist.org/clk/pts/d/vancouver-new-pair-tesla-model-front/7908199617.html</t>
+          <t>https://seattle.craigslist.org/skc/pts/d/seattle-tesla-model-clear-ppf-hood/7917727783.html</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:31+00:00</t>
+          <t>2026-05-01T11:36:30+00:00</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -10533,17 +10533,17 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Tesla Model 3 Clear PPF Hood, fenders, headlights, mirrors fog lights</t>
+          <t>NEW 2017 2022 2023 Pair TESLA MODEL 3 FRONT LEFT RIGHT Side HOOD HINGE</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>$229</t>
+          <t>$80</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>portland / Tukwila</t>
+          <t>eugene / clark/cowlitz WA</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -10573,12 +10573,12 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/skc/pts/d/seattle-tesla-model-clear-ppf-hood/7917727783.html</t>
+          <t>https://portland.craigslist.org/clk/pts/d/vancouver-new-pair-tesla-model-front/7908199617.html</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:31+00:00</t>
+          <t>2026-05-01T11:36:34+00:00</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -10610,17 +10610,17 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>NEW 2017 2022 2023 Pair TESLA MODEL 3 FRONT LEFT RIGHT Side HOOD HINGE</t>
+          <t>Tesla Model 3 Clear PPF Hood, fenders, headlights, mirrors fog lights</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>$80</t>
+          <t>$229</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>eugene / clark/cowlitz WA</t>
+          <t>eugene / Tukwila</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -10650,12 +10650,12 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>https://portland.craigslist.org/clk/pts/d/vancouver-new-pair-tesla-model-front/7908199617.html</t>
+          <t>https://seattle.craigslist.org/skc/pts/d/seattle-tesla-model-clear-ppf-hood/7917727783.html</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:35+00:00</t>
+          <t>2026-05-01T11:36:34+00:00</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -10687,27 +10687,27 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Tesla Model 3 Clear PPF Hood, fenders, headlights, mirrors fog lights</t>
+          <t>Tesla model 3 or Y headlight Left side</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>$229</t>
+          <t>$350</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>eugene / Tukwila</t>
+          <t>bellingham / Milwaukie</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t> Tesla Model 3</t>
+          <t> Tesla Model Y</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>hood</t>
+          <t>headlight</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -10727,17 +10727,17 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/skc/pts/d/seattle-tesla-model-clear-ppf-hood/7917727783.html</t>
+          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-or-headlight-left/7929779630.html</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:35+00:00</t>
+          <t>2026-05-01T11:35:21+00:00</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>53</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
@@ -10752,7 +10752,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>year match, model match, part match, price visible, direct link, public source</t>
+          <t>year match, part match, price visible, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -10764,27 +10764,27 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>NEW 2017 2022 2023 Pair TESLA MODEL 3 FRONT LEFT RIGHT Side HOOD HINGE</t>
+          <t>Tesla model 3 or Y headlight Left side</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>$80</t>
+          <t>$350</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>bend / clark/cowlitz WA</t>
+          <t>portland / Milwaukie</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t> Tesla Model 3</t>
+          <t> Tesla Model Y</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>hood</t>
+          <t>headlight</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -10804,17 +10804,17 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>https://portland.craigslist.org/clk/pts/d/vancouver-new-pair-tesla-model-front/7908199617.html</t>
+          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-or-headlight-left/7929779630.html</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:39+00:00</t>
+          <t>2026-05-01T11:35:24+00:00</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>53</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
@@ -10829,7 +10829,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>year match, model match, part match, price visible, direct link, public source</t>
+          <t>year match, part match, price visible, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -10841,27 +10841,27 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Tesla Model 3 Clear PPF Hood, fenders, headlights, mirrors fog lights</t>
+          <t>Tesla model 3 or Y headlight Left side</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>$229</t>
+          <t>$350</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>bend / Tukwila</t>
+          <t>eugene / Milwaukie</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t> Tesla Model 3</t>
+          <t> Tesla Model Y</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>hood</t>
+          <t>headlight</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -10881,17 +10881,17 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/skc/pts/d/seattle-tesla-model-clear-ppf-hood/7917727783.html</t>
+          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-or-headlight-left/7929779630.html</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:39+00:00</t>
+          <t>2026-05-01T11:35:28+00:00</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>53</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
@@ -10906,7 +10906,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>year match, model match, part match, price visible, direct link, public source</t>
+          <t>year match, part match, price visible, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -10928,7 +10928,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>bellingham / Milwaukie</t>
+          <t>bend / Milwaukie</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -10963,7 +10963,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:19+00:00</t>
+          <t>2026-05-01T11:35:32+00:00</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -10995,17 +10995,17 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Tesla model 3 or Y headlight Left side</t>
+          <t>Tesla half yolk steering wheel</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>$350</t>
+          <t>$200</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>portland / Milwaukie</t>
+          <t>spokane / Seattle</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -11015,7 +11015,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>headlight</t>
+          <t>wheel</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -11035,12 +11035,12 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-or-headlight-left/7929779630.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/tesla-half-yolk-steering-wheel/7930743561.html</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:22+00:00</t>
+          <t>2026-05-01T11:36:02+00:00</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -11072,17 +11072,17 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Tesla model 3 or Y headlight Left side</t>
+          <t>Tesla half yolk steering wheel</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>$350</t>
+          <t>$200</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>eugene / Milwaukie</t>
+          <t>portland / Seattle</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -11092,7 +11092,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>headlight</t>
+          <t>wheel</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -11112,12 +11112,12 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-or-headlight-left/7929779630.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/tesla-half-yolk-steering-wheel/7930743561.html</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:25+00:00</t>
+          <t>2026-05-01T11:36:10+00:00</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -11149,17 +11149,17 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Tesla model 3 or Y headlight Left side</t>
+          <t>Tesla half yolk steering wheel</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>$350</t>
+          <t>$200</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>bend / Milwaukie</t>
+          <t>eugene / Seattle</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -11169,7 +11169,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>headlight</t>
+          <t>wheel</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -11189,12 +11189,12 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>https://portland.craigslist.org/mlt/pts/d/portland-tesla-model-or-headlight-left/7929779630.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/tesla-half-yolk-steering-wheel/7930743561.html</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:29+00:00</t>
+          <t>2026-05-01T11:36:14+00:00</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
@@ -11226,17 +11226,17 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Tesla half yolk steering wheel</t>
+          <t>Tesla Model Y 3 Parts</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>$200</t>
+          <t/>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>spokane / Seattle</t>
+          <t>spokane / Marysville</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -11246,7 +11246,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>wheel</t>
+          <t>front bumper</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -11266,17 +11266,17 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/see/pts/d/tesla-half-yolk-steering-wheel/7930743561.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-3-parts/7921311562.html</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>2026-05-01T09:54:58+00:00</t>
+          <t>2026-05-01T11:34:21+00:00</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>43</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
@@ -11291,7 +11291,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>year match, part match, price visible, direct link, public source</t>
+          <t>year match, model match, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -11303,17 +11303,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Tesla half yolk steering wheel</t>
+          <t>Tesla Model Y 3 Parts</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>$200</t>
+          <t/>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>portland / Seattle</t>
+          <t>bellingham / Marysville</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -11323,7 +11323,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>wheel</t>
+          <t>front bumper</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -11343,17 +11343,17 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/see/pts/d/tesla-half-yolk-steering-wheel/7930743561.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-3-parts/7921311562.html</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:08+00:00</t>
+          <t>2026-05-01T11:34:25+00:00</t>
         </is>
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>43</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>year match, part match, price visible, direct link, public source</t>
+          <t>year match, model match, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -11380,17 +11380,17 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Tesla half yolk steering wheel</t>
+          <t>Tesla Model Y 3 Parts</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>$200</t>
+          <t/>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>eugene / Seattle</t>
+          <t>portland / Marysville</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -11400,7 +11400,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>wheel</t>
+          <t>front bumper</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -11420,17 +11420,17 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/see/pts/d/tesla-half-yolk-steering-wheel/7930743561.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-3-parts/7921311562.html</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:11+00:00</t>
+          <t>2026-05-01T11:34:29+00:00</t>
         </is>
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>43</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
@@ -11445,7 +11445,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>year match, part match, price visible, direct link, public source</t>
+          <t>year match, model match, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -11457,17 +11457,17 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Tesla half yolk steering wheel</t>
+          <t>Tesla Model Y 3 Parts</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>$200</t>
+          <t/>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>bend / Seattle</t>
+          <t>seattle / Marysville</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -11477,7 +11477,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>wheel</t>
+          <t>rear bumper</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -11497,17 +11497,17 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>https://seattle.craigslist.org/see/pts/d/tesla-half-yolk-steering-wheel/7930743561.html</t>
+          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-3-parts/7921311562.html</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:14+00:00</t>
+          <t>2026-05-01T11:34:54+00:00</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>43</t>
         </is>
       </c>
       <c r="M149" t="inlineStr">
@@ -11522,7 +11522,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>year match, part match, price visible, direct link, public source</t>
+          <t>year match, model match, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -11544,7 +11544,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>bellingham / Marysville</t>
+          <t>spokane / Marysville</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -11554,7 +11554,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>front bumper</t>
+          <t>rear bumper</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -11579,7 +11579,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:35+00:00</t>
+          <t>2026-05-01T11:34:57+00:00</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -11621,7 +11621,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>portland / Marysville</t>
+          <t>bellingham / Marysville</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>front bumper</t>
+          <t>rear bumper</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -11656,7 +11656,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:38+00:00</t>
+          <t>2026-05-01T11:35:01+00:00</t>
         </is>
       </c>
       <c r="L151" t="inlineStr">
@@ -11698,7 +11698,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>seattle / Marysville</t>
+          <t>portland / Marysville</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -11733,7 +11733,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:49+00:00</t>
+          <t>2026-05-01T11:35:04+00:00</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
@@ -11775,17 +11775,17 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>bellingham / Marysville</t>
+          <t>seattle / Marysville</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t> Tesla Model Y</t>
+          <t> Tesla Model 3</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>rear bumper</t>
+          <t>front bumper</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -11810,12 +11810,12 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:55+00:00</t>
+          <t>2026-05-01T11:36:42+00:00</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>23</t>
         </is>
       </c>
       <c r="M153" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>year match, model match, direct link, public source</t>
+          <t>year match, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -11852,17 +11852,17 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>portland / Marysville</t>
+          <t>spokane / Marysville</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t> Tesla Model Y</t>
+          <t> Tesla Model 3</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>rear bumper</t>
+          <t>front bumper</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -11887,12 +11887,12 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>2026-05-01T09:53:58+00:00</t>
+          <t>2026-05-01T11:36:48+00:00</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>23</t>
         </is>
       </c>
       <c r="M154" t="inlineStr">
@@ -11907,7 +11907,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>year match, model match, direct link, public source</t>
+          <t>year match, direct link, public source</t>
         </is>
       </c>
     </row>
@@ -11929,7 +11929,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>spokane / Marysville</t>
+          <t>portland / Marysville</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -11964,7 +11964,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>2026-05-01T09:55:48+00:00</t>
+          <t>2026-05-01T11:36:55+00:00</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
@@ -11983,160 +11983,6 @@
         </is>
       </c>
       <c r="O155" t="inlineStr">
-        <is>
-          <t>year match, direct link, public source</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>Tesla Model Y 3 Parts</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>bellingham / Marysville</t>
-        </is>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t> Tesla Model 3</t>
-        </is>
-      </c>
-      <c r="F156" t="inlineStr">
-        <is>
-          <t>front bumper</t>
-        </is>
-      </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I156" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J156" t="inlineStr">
-        <is>
-          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-3-parts/7921311562.html</t>
-        </is>
-      </c>
-      <c r="K156" t="inlineStr">
-        <is>
-          <t>2026-05-01T09:55:52+00:00</t>
-        </is>
-      </c>
-      <c r="L156" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="M156" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N156" t="inlineStr">
-        <is>
-          <t>Duplicate</t>
-        </is>
-      </c>
-      <c r="O156" t="inlineStr">
-        <is>
-          <t>year match, direct link, public source</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>Craigslist</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>Tesla Model Y 3 Parts</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>portland / Marysville</t>
-        </is>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t> Tesla Model 3</t>
-        </is>
-      </c>
-      <c r="F157" t="inlineStr">
-        <is>
-          <t>front bumper</t>
-        </is>
-      </c>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H157" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I157" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J157" t="inlineStr">
-        <is>
-          <t>https://seattle.craigslist.org/see/pts/d/marysville-tesla-model-3-parts/7921311562.html</t>
-        </is>
-      </c>
-      <c r="K157" t="inlineStr">
-        <is>
-          <t>2026-05-01T09:55:55+00:00</t>
-        </is>
-      </c>
-      <c r="L157" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="M157" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N157" t="inlineStr">
-        <is>
-          <t>Duplicate</t>
-        </is>
-      </c>
-      <c r="O157" t="inlineStr">
         <is>
           <t>year match, direct link, public source</t>
         </is>

</xml_diff>